<commit_message>
Corrections apportées suite aux reviews fc2b6baf6dbe4268980b02ef2522147e1961d7f1
</commit_message>
<xml_diff>
--- a/HTR-IGDoc/ig/StructureDefinition-fr-core-service-event.xlsx
+++ b/HTR-IGDoc/ig/StructureDefinition-fr-core-service-event.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-24T14:08:41+00:00</t>
+    <t>2025-02-25T09:00:30+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -449,7 +449,7 @@
 - Pour un document au format CDA R2 N3, se reporter au volet de contenus correspondant.
 - Pour certains documents au format CDA R2 N1, la valeur est fixée (voir tableau qui suit).
 - Dans les autres cas, utiliser une valeur issue d'une terminologie internationale (ex : CIM10 pour les actes) ou nationale (ex : CCAM pour les actes).
-Pour les documents d’expression personnelle du patient/usager :
+- Pour les documents d’expression personnelle du patient/usager :
 - valeur fixée</t>
   </si>
   <si>

</xml_diff>